<commit_message>
update to vegetation data cleaning and analysis
</commit_message>
<xml_diff>
--- a/data/processed/LP_R&S_C123_Yr1-5_PSU_Sampled.xlsx
+++ b/data/processed/LP_R&S_C123_Yr1-5_PSU_Sampled.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fiudit-my.sharepoint.com/personal/gannd_fiu_edu/Documents/2_dev/_git_repo/LPstatreview/20260216_LPstatReview/data/processed/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fiudit-my.sharepoint.com/personal/gannd_fiu_edu/Documents/2_dev/_git_repo/LPstatreview/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{5244B2A3-2B5A-40F5-B89B-6CA7B7F83BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3050F6B5-72F3-47E5-9824-BD1728D0AD26}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{5244B2A3-2B5A-40F5-B89B-6CA7B7F83BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59C21836-8B51-4090-9EFD-FADCF2CCB42E}"/>
   <bookViews>
-    <workbookView xWindow="1365" yWindow="-19185" windowWidth="31740" windowHeight="18855" xr2:uid="{9DC1F7AA-CC20-40AC-B2AE-F561414E351E}"/>
+    <workbookView xWindow="13710" yWindow="-17115" windowWidth="23475" windowHeight="16530" xr2:uid="{9DC1F7AA-CC20-40AC-B2AE-F561414E351E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1522,6 +1522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA7695F7-AB8D-4AA7-9F38-E42449A2BF73}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:V69"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1613,7 +1614,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>9</v>
       </c>
@@ -1678,7 +1679,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>14</v>
       </c>
@@ -1743,7 +1744,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
@@ -1808,7 +1809,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>19</v>
       </c>
@@ -1873,7 +1874,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>21</v>
       </c>
@@ -1938,7 +1939,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>23</v>
       </c>
@@ -2003,7 +2004,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>25</v>
       </c>
@@ -2068,7 +2069,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -2133,7 +2134,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>29</v>
       </c>
@@ -2198,7 +2199,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -2263,7 +2264,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>33</v>
       </c>
@@ -2393,7 +2394,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -2458,7 +2459,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>39</v>
       </c>
@@ -2523,7 +2524,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>41</v>
       </c>
@@ -2588,7 +2589,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
         <v>43</v>
       </c>
@@ -2653,7 +2654,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="18" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>44</v>
       </c>
@@ -2718,7 +2719,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="9" t="s">
         <v>46</v>
       </c>
@@ -2783,7 +2784,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>48</v>
       </c>
@@ -2848,7 +2849,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>51</v>
       </c>
@@ -2913,7 +2914,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="22" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>52</v>
       </c>
@@ -2978,7 +2979,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="s">
         <v>54</v>
       </c>
@@ -3043,7 +3044,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
         <v>56</v>
       </c>
@@ -3173,7 +3174,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="9" t="s">
         <v>59</v>
       </c>
@@ -3303,7 +3304,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="28" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="s">
         <v>63</v>
       </c>
@@ -3433,7 +3434,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="9" t="s">
         <v>66</v>
       </c>
@@ -3498,7 +3499,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="9" t="s">
         <v>68</v>
       </c>
@@ -3563,7 +3564,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="9" t="s">
         <v>70</v>
       </c>
@@ -3628,7 +3629,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="33" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="s">
         <v>72</v>
       </c>
@@ -3693,7 +3694,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="34" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="s">
         <v>74</v>
       </c>
@@ -3758,7 +3759,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="35" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="9" t="s">
         <v>75</v>
       </c>
@@ -3823,7 +3824,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="36" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="9" t="s">
         <v>77</v>
       </c>
@@ -3888,7 +3889,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="37" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="9" t="s">
         <v>79</v>
       </c>
@@ -3953,7 +3954,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="38" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="s">
         <v>81</v>
       </c>
@@ -4018,7 +4019,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="39" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="s">
         <v>83</v>
       </c>
@@ -4083,7 +4084,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="40" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="9" t="s">
         <v>85</v>
       </c>
@@ -4148,7 +4149,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="9" t="s">
         <v>87</v>
       </c>
@@ -4213,7 +4214,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="42" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="9" t="s">
         <v>89</v>
       </c>
@@ -4278,7 +4279,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="43" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="s">
         <v>91</v>
       </c>
@@ -4343,7 +4344,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="s">
         <v>93</v>
       </c>
@@ -4408,7 +4409,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="45" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="s">
         <v>95</v>
       </c>
@@ -4473,7 +4474,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="46" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
         <v>97</v>
       </c>
@@ -4538,7 +4539,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="47" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="s">
         <v>99</v>
       </c>
@@ -4603,7 +4604,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="48" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="s">
         <v>101</v>
       </c>
@@ -4668,7 +4669,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="49" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
         <v>103</v>
       </c>
@@ -4733,7 +4734,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="50" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
         <v>194</v>
       </c>
@@ -4798,7 +4799,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="51" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
         <v>105</v>
       </c>
@@ -4863,7 +4864,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="52" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
         <v>107</v>
       </c>
@@ -4928,7 +4929,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="s">
         <v>109</v>
       </c>
@@ -4993,7 +4994,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="54" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="9" t="s">
         <v>111</v>
       </c>
@@ -5059,7 +5060,7 @@
       </c>
       <c r="V54" s="2"/>
     </row>
-    <row r="55" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
         <v>113</v>
       </c>
@@ -5125,7 +5126,7 @@
       </c>
       <c r="V55" s="2"/>
     </row>
-    <row r="56" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="9" t="s">
         <v>115</v>
       </c>
@@ -5191,7 +5192,7 @@
       </c>
       <c r="V56" s="2"/>
     </row>
-    <row r="57" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="s">
         <v>117</v>
       </c>
@@ -5257,7 +5258,7 @@
       </c>
       <c r="V57" s="2"/>
     </row>
-    <row r="58" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="9" t="s">
         <v>119</v>
       </c>
@@ -5323,7 +5324,7 @@
       </c>
       <c r="V58" s="2"/>
     </row>
-    <row r="59" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
         <v>121</v>
       </c>
@@ -5389,7 +5390,7 @@
       </c>
       <c r="V59" s="2"/>
     </row>
-    <row r="60" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
         <v>123</v>
       </c>
@@ -5455,7 +5456,7 @@
       </c>
       <c r="V60" s="2"/>
     </row>
-    <row r="61" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="9" t="s">
         <v>125</v>
       </c>
@@ -5521,7 +5522,7 @@
       </c>
       <c r="V61" s="2"/>
     </row>
-    <row r="62" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="9" t="s">
         <v>127</v>
       </c>
@@ -5587,7 +5588,7 @@
       </c>
       <c r="V62" s="2"/>
     </row>
-    <row r="63" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="9" t="s">
         <v>129</v>
       </c>
@@ -5653,7 +5654,7 @@
       </c>
       <c r="V63" s="2"/>
     </row>
-    <row r="64" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="9" t="s">
         <v>131</v>
       </c>
@@ -5719,7 +5720,7 @@
       </c>
       <c r="V64" s="2"/>
     </row>
-    <row r="65" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="9" t="s">
         <v>133</v>
       </c>
@@ -5785,7 +5786,7 @@
       </c>
       <c r="V65" s="2"/>
     </row>
-    <row r="66" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="9" t="s">
         <v>136</v>
       </c>
@@ -5850,7 +5851,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="67" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="9" t="s">
         <v>139</v>
       </c>
@@ -5915,7 +5916,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="68" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="9" t="s">
         <v>142</v>
       </c>
@@ -5985,7 +5986,16 @@
       <c r="F69" s="30"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U68" xr:uid="{AA7695F7-AB8D-4AA7-9F38-E42449A2BF73}"/>
+  <autoFilter ref="A1:U68" xr:uid="{AA7695F7-AB8D-4AA7-9F38-E42449A2BF73}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="13"/>
+        <filter val="25"/>
+        <filter val="27"/>
+        <filter val="29"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>